<commit_message>
docs(template): thêm ward_code, ward_name, bc_giao_name vào template đổi kho
Sheet 'Template nhập' bổ sung 3 cột: mã phường, tên phường, tên BC giao.
Cập nhật COUNTIFS bảng lý do (ly_do_code dời sang cột J).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Template_Ly_Do_Doi_Kho.xlsx
+++ b/templates/Template_Ly_Do_Doi_Kho.xlsx
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -556,9 +556,12 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -571,7 +574,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mỗi đơn bị đổi kho giao là 1 dòng. Bảng 'Lý do đổi kho' sẽ tự tính từ dữ liệu ở đây (COUNTIFS). Nhập từ dòng 4.</t>
+          <t>Mỗi đơn bị đổi kho giao là 1 dòng. Bảng 'Lý do đổi kho' tự tính từ dữ liệu ở đây (COUNTIFS theo channel/phường/lý do). Nhập từ dòng 5.</t>
         </is>
       </c>
     </row>
@@ -603,15 +606,30 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
+          <t>ward_code</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>ward_name</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>bc_giao_code</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>bc_giao_name</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>ly_do_code</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>ghi_chu</t>
         </is>
@@ -645,15 +663,30 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
+          <t>Mã phường (ward code)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Tên phường (ward name)</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
           <t>Mã BC giao</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Tên BC giao</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Mã lý do (xem sheet Mã lý do)</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Ghi chú (tuỳ chọn)</t>
         </is>
@@ -685,15 +718,30 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
+          <t>26737</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Phường Bến Thành</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
           <t>BC-HCM-007</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>BC TP.HCM 007 (Q1)</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>routing-rule</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr"/>
+      <c r="K5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -721,15 +769,30 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
+          <t>26773</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Phường Đa Kao</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
           <t>BC-HCM-012</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>BC TP.HCM 012 (Q1)</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>address-error</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr"/>
+      <c r="K6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -757,15 +820,30 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
+          <t>27154</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Phường 12 (Bình Thạnh)</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
           <t>BC-HCM-003</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>BC TP.HCM 003 (Bình Thạnh)</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>bc-closed</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr"/>
+      <c r="K7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -793,15 +871,30 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
+          <t>00037</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Phường Trúc Bạch</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
           <t>BC-HNI-021</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>BC Hà Nội 021 (Ba Đình)</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>routing-rule</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr"/>
+      <c r="K8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -829,15 +922,30 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
+          <t>00103</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Phường Hàng Bạc</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
           <t>BC-HNI-005</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>BC Hà Nội 005 (Hoàn Kiếm)</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>bc-closed</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr"/>
+      <c r="K9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -865,15 +973,30 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
+          <t>00148</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Phường Cát Linh</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
           <t>BC-HNI-008</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>BC Hà Nội 008 (Đống Đa)</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>service-unavail</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr"/>
+      <c r="K10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -901,15 +1024,30 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
+          <t>11401</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Phường Máy Chai</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
           <t>BC-HPG-002</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>BC Hải Phòng 002 (Ngô Quyền)</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>address-error</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr"/>
+      <c r="K11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -937,15 +1075,30 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
+          <t>11428</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Phường Cầu Đất</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
           <t>BC-HPG-009</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>BC Hải Phòng 009 (Lê Chân)</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>routing-rule</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr"/>
+      <c r="K12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -973,15 +1126,30 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
+          <t>11461</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Phường Anh Dũng</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
           <t>BC-HPG-004</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>BC Hải Phòng 004 (Dương Kinh)</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>bc-closed</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr"/>
+      <c r="K13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1009,15 +1177,30 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
+          <t>27190</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Phường 5 (Gò Vấp)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
           <t>BC-HCM-015</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>BC TP.HCM 015 (Gò Vấp)</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>khac</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr"/>
+      <c r="K14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1045,15 +1228,30 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
+          <t>00220</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Phường Dịch Vọng</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
           <t>BC-HNI-011</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>BC Hà Nội 011 (Cầu Giấy)</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>address-error</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr"/>
+      <c r="K15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1081,15 +1279,30 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
+          <t>25744</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Phường Phú Lợi</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
           <t>BC-BDG-006</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>BC Bình Dương 006 (Thủ Dầu Một)</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>service-unavail</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr"/>
+      <c r="K16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1117,15 +1330,30 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
+          <t>27001</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Phường Tân Định</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
           <t>BC-HCM-020</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>BC TP.HCM 020 (Q1)</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>routing-rule</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr"/>
+      <c r="K17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1153,15 +1381,30 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
+          <t>27259</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Phường 15 (Tân Bình)</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
           <t>BC-HCM-031</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>BC TP.HCM 031 (Tân Bình)</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>bc-closed</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr"/>
+      <c r="K18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1189,15 +1432,30 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
+          <t>00271</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Phường Nghĩa Đô</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
           <t>BC-HNI-014</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>BC Hà Nội 014 (Cầu Giấy)</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>routing-rule</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr"/>
+      <c r="K19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1225,15 +1483,30 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
+          <t>11503</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Phường Hùng Vương</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
           <t>BC-HPG-012</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>BC Hải Phòng 012 (Hồng Bàng)</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>khac</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr"/>
+      <c r="K20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1261,15 +1534,30 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
+          <t>26821</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Phường Cô Giang</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
           <t>BC-HCM-008</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>BC TP.HCM 008 (Q1)</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
         <is>
           <t>address-error</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr"/>
+      <c r="K21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1297,15 +1585,30 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
+          <t>00316</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Phường Phúc Xá</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
           <t>BC-HNI-019</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>BC Hà Nội 019 (Ba Đình)</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>bc-closed</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr"/>
+      <c r="K22" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1343,7 +1646,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tự tính từ sheet 'Template nhập'. Mỗi cột (Nguồn × Mới/Cũ) cộng các lý do = 100%. Phường mới thường lệch về sai routing/mapping; phường cũ về BC đóng/quá tải.</t>
+          <t>Tự tính từ sheet 'Template nhập'. Mỗi cột (Nguồn × Mới/Cũ) cộng các lý do = 100%.</t>
         </is>
       </c>
     </row>
@@ -1433,35 +1736,35 @@
         </is>
       </c>
       <c r="B6" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K6)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K6)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="C6" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K6)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K6)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="D6" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="E6" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="F6" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="G6" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="H6" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="I6" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K6)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="K6" s="15" t="inlineStr">
@@ -1477,35 +1780,35 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K7)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K7)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="C7" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K7)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K7)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="D7" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="E7" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="F7" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="G7" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="H7" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="I7" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K7)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="K7" s="15" t="inlineStr">
@@ -1521,35 +1824,35 @@
         </is>
       </c>
       <c r="B8" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K8)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K8)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="C8" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K8)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K8)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="D8" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="E8" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="F8" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="G8" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="H8" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="I8" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K8)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="K8" s="15" t="inlineStr">
@@ -1565,35 +1868,35 @@
         </is>
       </c>
       <c r="B9" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K9)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K9)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="C9" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K9)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K9)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="D9" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="E9" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="F9" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="G9" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="H9" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="I9" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K9)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="K9" s="15" t="inlineStr">
@@ -1609,35 +1912,35 @@
         </is>
       </c>
       <c r="B10" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K10)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K10)/COUNTIFS('Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="C10" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K10)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K10)/COUNTIFS('Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="D10" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="E10" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"spe",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="F10" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="G10" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"tts",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="H10" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$G$5:$G$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1,'Template nhập'!$J$5:$J$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,1),0)</f>
         <v/>
       </c>
       <c r="I10" s="14">
-        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$G$5:$G$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
+        <f>IFERROR(COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0,'Template nhập'!$J$5:$J$1000,$K10)/COUNTIFS('Template nhập'!$C$5:$C$1000,"sme",'Template nhập'!$D$5:$D$1000,0),0)</f>
         <v/>
       </c>
       <c r="K10" s="15" t="inlineStr">
@@ -1869,7 +2172,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1882,7 +2185,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tổng hợp sẵn theo ngày × nguồn × phường × lý do. Cột so_don = số đơn đổi kho của tổ hợp đó.</t>
+          <t>Tổng hợp sẵn theo ngày × nguồn × phường × lý do. so_don = số đơn đổi kho của tổ hợp.</t>
         </is>
       </c>
     </row>
@@ -1916,7 +2219,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Ngày (yyyy-mm-dd)</t>
+          <t>Ngày</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1926,7 +2229,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1=mới, 0=cũ</t>
+          <t>1=mới,0=cũ</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1936,7 +2239,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Số đơn đổi kho</t>
+          <t>Số đơn</t>
         </is>
       </c>
     </row>

</xml_diff>